<commit_message>
Changes to new maps
</commit_message>
<xml_diff>
--- a/FinalSheet.xlsx
+++ b/FinalSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nehakotha/GASP-Clean-Air-Fund/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2C79A08-BCA3-F044-8390-49A5E4EF578C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2460930-DE11-E743-BC94-3E5522919E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6880" yWindow="760" windowWidth="23360" windowHeight="16300" xr2:uid="{C5E92D08-1D1E-B946-9078-11755ACCCC10}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="64">
   <si>
     <t>Year</t>
   </si>
@@ -116,9 +116,6 @@
     <t>Solarize Allegheny</t>
   </si>
   <si>
-    <t>Southwest Pennsylvania Air Quality</t>
-  </si>
-  <si>
     <t>Pittsburgh</t>
   </si>
   <si>
@@ -137,21 +134,12 @@
     <t>enfoTech &amp; Consulting Inc.</t>
   </si>
   <si>
-    <t xml:space="preserve">Steel Rivers Council of Governments </t>
-  </si>
-  <si>
     <t>West Mifflin Borough</t>
   </si>
   <si>
     <t>Wilkinsburg Shade Tree Commission</t>
   </si>
   <si>
-    <t>Brackenridge</t>
-  </si>
-  <si>
-    <t>Pitcairn</t>
-  </si>
-  <si>
     <t>Munhall Borough</t>
   </si>
   <si>
@@ -231,6 +219,15 @@
   </si>
   <si>
     <t>…..</t>
+  </si>
+  <si>
+    <t>Steel Rivers Council of Governments</t>
+  </si>
+  <si>
+    <t>Air Quality Program+G15</t>
+  </si>
+  <si>
+    <t>Several small projects</t>
   </si>
 </sst>
 </file>
@@ -319,7 +316,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -382,6 +379,11 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -754,13 +756,13 @@
         <v>11</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="G1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="H1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -780,13 +782,13 @@
         <v>12</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="H2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -806,13 +808,13 @@
         <v>12</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G3" s="15" t="s">
         <v>22</v>
       </c>
       <c r="H3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I3" s="4"/>
     </row>
@@ -839,7 +841,7 @@
         <v>3</v>
       </c>
       <c r="H4" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I4" s="21"/>
     </row>
@@ -860,13 +862,13 @@
         <v>12</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="G5" s="15" t="s">
         <v>23</v>
       </c>
       <c r="H5" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I5" s="4"/>
     </row>
@@ -887,13 +889,13 @@
         <v>16</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="H6" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I6" s="7"/>
     </row>
@@ -920,7 +922,7 @@
         <v>6</v>
       </c>
       <c r="H7" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I7" s="4"/>
     </row>
@@ -943,11 +945,11 @@
       <c r="F8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="15" t="s">
+      <c r="G8" s="24" t="s">
         <v>9</v>
       </c>
       <c r="H8" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I8" s="4"/>
     </row>
@@ -968,13 +970,13 @@
         <v>12</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="G9" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G9" s="24" t="s">
         <v>24</v>
       </c>
       <c r="H9" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I9" s="4"/>
     </row>
@@ -997,11 +999,11 @@
       <c r="F10" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="15" t="s">
+      <c r="G10" s="24" t="s">
         <v>25</v>
       </c>
       <c r="H10" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I10" s="7"/>
     </row>
@@ -1024,11 +1026,11 @@
       <c r="F11" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="15" t="s">
+      <c r="G11" s="24" t="s">
         <v>3</v>
       </c>
       <c r="H11" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I11" s="7"/>
     </row>
@@ -1051,11 +1053,11 @@
       <c r="F12" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="15" t="s">
-        <v>26</v>
+      <c r="G12" s="24" t="s">
+        <v>4</v>
       </c>
       <c r="H12" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I12" s="7"/>
     </row>
@@ -1076,13 +1078,13 @@
         <v>12</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
+      </c>
+      <c r="G13" s="25" t="s">
+        <v>38</v>
       </c>
       <c r="H13" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1104,11 +1106,11 @@
       <c r="F14" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="15" t="s">
+      <c r="G14" s="24" t="s">
         <v>3</v>
       </c>
       <c r="H14" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I14" s="4"/>
     </row>
@@ -1129,13 +1131,13 @@
         <v>12</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G15" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="G15" s="24" t="s">
         <v>7</v>
       </c>
       <c r="H15" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I15" s="4"/>
     </row>
@@ -1162,7 +1164,7 @@
         <v>9</v>
       </c>
       <c r="H16" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1188,7 +1190,7 @@
         <v>6</v>
       </c>
       <c r="H17" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I17" s="7"/>
     </row>
@@ -1212,10 +1214,10 @@
         <v>5</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H18" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I18" s="7"/>
     </row>
@@ -1242,7 +1244,7 @@
         <v>6</v>
       </c>
       <c r="H19" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I19" s="22"/>
     </row>
@@ -1269,7 +1271,7 @@
         <v>6</v>
       </c>
       <c r="H20" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I20" s="4"/>
     </row>
@@ -1296,7 +1298,7 @@
         <v>6</v>
       </c>
       <c r="H21" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I21" s="4"/>
     </row>
@@ -1323,7 +1325,7 @@
         <v>6</v>
       </c>
       <c r="H22" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I22" s="4"/>
     </row>
@@ -1350,7 +1352,7 @@
         <v>6</v>
       </c>
       <c r="H23" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I23" s="4"/>
     </row>
@@ -1377,7 +1379,7 @@
         <v>6</v>
       </c>
       <c r="H24" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I24" s="4"/>
     </row>
@@ -1404,7 +1406,7 @@
         <v>6</v>
       </c>
       <c r="H25" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I25" s="4"/>
     </row>
@@ -1431,7 +1433,7 @@
         <v>6</v>
       </c>
       <c r="H26" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I26" s="5"/>
     </row>
@@ -1455,10 +1457,10 @@
         <v>5</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H27" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I27" s="8"/>
     </row>
@@ -1482,10 +1484,10 @@
         <v>5</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="H28" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I28" s="5"/>
     </row>
@@ -1506,13 +1508,13 @@
         <v>12</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="G29" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H29" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I29" s="5"/>
     </row>
@@ -1533,13 +1535,13 @@
         <v>12</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G30" s="15" t="s">
         <v>3</v>
       </c>
       <c r="H30" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I30" s="8"/>
     </row>
@@ -1562,11 +1564,11 @@
       <c r="F31" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="14" t="s">
+      <c r="G31" s="26" t="s">
         <v>4</v>
       </c>
       <c r="H31" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I31" s="4"/>
     </row>
@@ -1587,13 +1589,13 @@
         <v>12</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
+      </c>
+      <c r="G32" s="25" t="s">
+        <v>38</v>
       </c>
       <c r="H32" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I32" s="5"/>
     </row>
@@ -1614,13 +1616,13 @@
         <v>12</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
+      </c>
+      <c r="G33" s="25" t="s">
+        <v>38</v>
       </c>
       <c r="H33" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I33" s="5"/>
     </row>
@@ -1643,11 +1645,11 @@
       <c r="F34" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G34" s="15" t="s">
+      <c r="G34" s="24" t="s">
         <v>6</v>
       </c>
       <c r="H34" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I34" s="5"/>
     </row>
@@ -1671,10 +1673,10 @@
         <v>5</v>
       </c>
       <c r="G35" s="15" t="s">
-        <v>6</v>
+        <v>62</v>
       </c>
       <c r="H35" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I35" s="5"/>
     </row>
@@ -1701,7 +1703,7 @@
         <v>6</v>
       </c>
       <c r="H36" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I36" s="5"/>
     </row>
@@ -1728,7 +1730,7 @@
         <v>6</v>
       </c>
       <c r="H37" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I37" s="8"/>
     </row>
@@ -1749,13 +1751,13 @@
         <v>12</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H38" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I38" s="5"/>
     </row>
@@ -1776,13 +1778,13 @@
         <v>12</v>
       </c>
       <c r="F39" s="23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H39" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I39" s="5"/>
     </row>
@@ -1809,7 +1811,7 @@
         <v>6</v>
       </c>
       <c r="H40" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I40" s="5"/>
     </row>
@@ -1836,7 +1838,7 @@
         <v>6</v>
       </c>
       <c r="H41" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I41" s="5"/>
     </row>
@@ -1860,10 +1862,10 @@
         <v>5</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H42" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I42" s="5"/>
     </row>
@@ -1890,7 +1892,7 @@
         <v>6</v>
       </c>
       <c r="H43" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I43" s="5"/>
     </row>
@@ -1911,13 +1913,13 @@
         <v>8</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="G44" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="G44" s="24" t="s">
         <v>22</v>
       </c>
       <c r="H44" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I44" s="5"/>
     </row>
@@ -1938,13 +1940,13 @@
         <v>12</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
+      </c>
+      <c r="G45" s="25" t="s">
+        <v>38</v>
       </c>
       <c r="H45" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I45" s="5"/>
     </row>
@@ -1965,13 +1967,13 @@
         <v>12</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="G46" s="15" t="s">
-        <v>31</v>
+        <v>26</v>
+      </c>
+      <c r="G46" s="24" t="s">
+        <v>30</v>
       </c>
       <c r="H46" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I46" s="5"/>
     </row>
@@ -1994,11 +1996,11 @@
       <c r="F47" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G47" s="15" t="s">
+      <c r="G47" s="24" t="s">
         <v>3</v>
       </c>
       <c r="H47" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I47" s="5"/>
     </row>
@@ -2021,11 +2023,11 @@
       <c r="F48" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G48" s="15" t="s">
+      <c r="G48" s="24" t="s">
         <v>3</v>
       </c>
       <c r="H48" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I48" s="5"/>
     </row>
@@ -2048,11 +2050,11 @@
       <c r="F49" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G49" s="14" t="s">
+      <c r="G49" s="26" t="s">
         <v>4</v>
       </c>
       <c r="H49" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I49" s="5"/>
     </row>
@@ -2075,11 +2077,11 @@
       <c r="F50" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G50" s="15" t="s">
+      <c r="G50" s="24" t="s">
         <v>3</v>
       </c>
       <c r="H50" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I50" s="5"/>
     </row>
@@ -2102,11 +2104,11 @@
       <c r="F51" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G51" s="15" t="s">
-        <v>32</v>
+      <c r="G51" s="24" t="s">
+        <v>31</v>
       </c>
       <c r="H51" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I51" s="23"/>
     </row>
@@ -2127,13 +2129,13 @@
         <v>12</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G52" s="16" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="H52" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I52" s="23"/>
     </row>
@@ -2154,13 +2156,13 @@
         <v>12</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G53" s="14" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="H53" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I53" s="23"/>
     </row>
@@ -2181,13 +2183,13 @@
         <v>12</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G54" s="15" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="H54" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I54" s="23"/>
     </row>
@@ -2208,13 +2210,13 @@
         <v>12</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="H55" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I55" s="5"/>
     </row>
@@ -2235,13 +2237,13 @@
         <v>12</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G56" s="15" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="H56" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I56" s="8"/>
     </row>
@@ -2262,13 +2264,13 @@
         <v>12</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G57" s="15" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="H57" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I57" s="20"/>
     </row>
@@ -2289,13 +2291,13 @@
         <v>12</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G58" s="15" t="s">
         <v>22</v>
       </c>
       <c r="H58" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I58" s="5"/>
     </row>
@@ -2316,13 +2318,13 @@
         <v>12</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G59" s="15" t="s">
         <v>22</v>
       </c>
       <c r="H59" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I59" s="5"/>
     </row>
@@ -2343,13 +2345,13 @@
         <v>12</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G60" s="15" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="H60" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I60" s="8"/>
     </row>
@@ -2370,13 +2372,13 @@
         <v>12</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="G61" s="15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H61" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I61" s="5"/>
     </row>
@@ -2397,13 +2399,13 @@
         <v>12</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G62" s="15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H62" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I62" s="5"/>
     </row>
@@ -2424,13 +2426,13 @@
         <v>12</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G63" s="15" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="H63" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I63" s="8"/>
     </row>
@@ -2451,13 +2453,13 @@
         <v>12</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="G64" s="15" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="H64" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I64" s="8"/>
     </row>
@@ -2478,13 +2480,13 @@
         <v>12</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="G65" s="20" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="H65" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I65" s="20"/>
     </row>
@@ -2505,13 +2507,13 @@
         <v>12</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G66" s="15" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="H66" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I66" s="8"/>
     </row>
@@ -2532,13 +2534,13 @@
         <v>12</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G67" s="15" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="H67" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I67" s="8"/>
     </row>
@@ -2559,13 +2561,13 @@
         <v>12</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G68" s="15" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="H68" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I68" s="8"/>
     </row>
@@ -2586,13 +2588,13 @@
         <v>12</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="G69" s="15" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="H69" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I69" s="8"/>
     </row>
@@ -2613,13 +2615,13 @@
         <v>15</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G70" s="15" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="H70" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I70" s="5"/>
     </row>

</xml_diff>

<commit_message>
changes to map viz
</commit_message>
<xml_diff>
--- a/FinalSheet.xlsx
+++ b/FinalSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nehakotha/GASP-Clean-Air-Fund/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2460930-DE11-E743-BC94-3E5522919E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4F87560-EB1C-9145-A172-4DC9CE4603A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6880" yWindow="760" windowWidth="23360" windowHeight="16300" xr2:uid="{C5E92D08-1D1E-B946-9078-11755ACCCC10}"/>
   </bookViews>
@@ -316,7 +316,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -379,11 +379,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -945,7 +940,7 @@
       <c r="F8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="24" t="s">
+      <c r="G8" s="15" t="s">
         <v>9</v>
       </c>
       <c r="H8" t="s">
@@ -972,7 +967,7 @@
       <c r="F9" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="G9" s="24" t="s">
+      <c r="G9" s="15" t="s">
         <v>24</v>
       </c>
       <c r="H9" t="s">
@@ -999,7 +994,7 @@
       <c r="F10" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="24" t="s">
+      <c r="G10" s="15" t="s">
         <v>25</v>
       </c>
       <c r="H10" t="s">
@@ -1026,7 +1021,7 @@
       <c r="F11" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="24" t="s">
+      <c r="G11" s="15" t="s">
         <v>3</v>
       </c>
       <c r="H11" t="s">
@@ -1053,7 +1048,7 @@
       <c r="F12" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="24" t="s">
+      <c r="G12" s="15" t="s">
         <v>4</v>
       </c>
       <c r="H12" t="s">
@@ -1080,7 +1075,7 @@
       <c r="F13" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G13" s="25" t="s">
+      <c r="G13" s="2" t="s">
         <v>38</v>
       </c>
       <c r="H13" t="s">
@@ -1106,7 +1101,7 @@
       <c r="F14" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="24" t="s">
+      <c r="G14" s="15" t="s">
         <v>3</v>
       </c>
       <c r="H14" t="s">
@@ -1133,7 +1128,7 @@
       <c r="F15" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G15" s="24" t="s">
+      <c r="G15" s="15" t="s">
         <v>7</v>
       </c>
       <c r="H15" t="s">
@@ -1564,7 +1559,7 @@
       <c r="F31" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="26" t="s">
+      <c r="G31" s="14" t="s">
         <v>4</v>
       </c>
       <c r="H31" t="s">
@@ -1591,7 +1586,7 @@
       <c r="F32" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G32" s="25" t="s">
+      <c r="G32" s="2" t="s">
         <v>38</v>
       </c>
       <c r="H32" t="s">
@@ -1618,7 +1613,7 @@
       <c r="F33" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G33" s="25" t="s">
+      <c r="G33" s="2" t="s">
         <v>38</v>
       </c>
       <c r="H33" t="s">
@@ -1645,7 +1640,7 @@
       <c r="F34" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G34" s="24" t="s">
+      <c r="G34" s="15" t="s">
         <v>6</v>
       </c>
       <c r="H34" t="s">
@@ -1915,7 +1910,7 @@
       <c r="F44" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="G44" s="24" t="s">
+      <c r="G44" s="15" t="s">
         <v>22</v>
       </c>
       <c r="H44" t="s">
@@ -1942,7 +1937,7 @@
       <c r="F45" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G45" s="25" t="s">
+      <c r="G45" s="2" t="s">
         <v>38</v>
       </c>
       <c r="H45" t="s">
@@ -1969,7 +1964,7 @@
       <c r="F46" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="G46" s="24" t="s">
+      <c r="G46" s="15" t="s">
         <v>30</v>
       </c>
       <c r="H46" t="s">
@@ -1996,7 +1991,7 @@
       <c r="F47" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G47" s="24" t="s">
+      <c r="G47" s="15" t="s">
         <v>3</v>
       </c>
       <c r="H47" t="s">
@@ -2023,7 +2018,7 @@
       <c r="F48" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G48" s="24" t="s">
+      <c r="G48" s="15" t="s">
         <v>3</v>
       </c>
       <c r="H48" t="s">
@@ -2050,7 +2045,7 @@
       <c r="F49" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G49" s="26" t="s">
+      <c r="G49" s="14" t="s">
         <v>4</v>
       </c>
       <c r="H49" t="s">
@@ -2077,7 +2072,7 @@
       <c r="F50" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G50" s="24" t="s">
+      <c r="G50" s="15" t="s">
         <v>3</v>
       </c>
       <c r="H50" t="s">
@@ -2104,7 +2099,7 @@
       <c r="F51" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G51" s="24" t="s">
+      <c r="G51" s="15" t="s">
         <v>31</v>
       </c>
       <c r="H51" t="s">

</xml_diff>

<commit_message>
changes to data and map
</commit_message>
<xml_diff>
--- a/FinalSheet.xlsx
+++ b/FinalSheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nehakotha/GASP-Clean-Air-Fund/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4F87560-EB1C-9145-A172-4DC9CE4603A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AA846D7-21B8-084C-89CD-7DADC50D572F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6880" yWindow="760" windowWidth="23360" windowHeight="16300" xr2:uid="{C5E92D08-1D1E-B946-9078-11755ACCCC10}"/>
+    <workbookView xWindow="6880" yWindow="4440" windowWidth="23360" windowHeight="16300" xr2:uid="{C5E92D08-1D1E-B946-9078-11755ACCCC10}"/>
   </bookViews>
   <sheets>
     <sheet name="FinalSheet" sheetId="4" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="130">
   <si>
     <t>Year</t>
   </si>
@@ -203,9 +203,6 @@
     <t>Allegheny County Parks Department</t>
   </si>
   <si>
-    <t>several small projects</t>
-  </si>
-  <si>
     <t>Lawrenceville, Chateau, Neville Island</t>
   </si>
   <si>
@@ -218,9 +215,6 @@
     <t>Project Description</t>
   </si>
   <si>
-    <t>…..</t>
-  </si>
-  <si>
     <t>Steel Rivers Council of Governments</t>
   </si>
   <si>
@@ -228,6 +222,237 @@
   </si>
   <si>
     <t>Several small projects</t>
+  </si>
+  <si>
+    <t>To support the Carnegie Science Center Future Cities Competition ($2,000 per year for 2015 and 2016).</t>
+  </si>
+  <si>
+    <t>To plant trees on industrial properties in Lawrenceville, Chateau, and Neville Island; requested by Tree Pittsburgh</t>
+  </si>
+  <si>
+    <t>To fund an outreach campaign in response to the revisions to Article XXI Open Burning regulations; the campaign will discourage open burning educate on the health effects of wood smoke</t>
+  </si>
+  <si>
+    <t>To support the Northgate Asthma Initiative / continue to concentrate the Healthy Homes program on children in the Northgate School District, which has an elevated number of asthmatic children</t>
+  </si>
+  <si>
+    <t>For the purchase of solar panels to light parking lots and charge electric vehicles at CCAC campuses.</t>
+  </si>
+  <si>
+    <t>To fund 50% of an investment-grade audit for renovation of Clack Building #1 as a potential new location for Air Quality.</t>
+  </si>
+  <si>
+    <t>To fund six Student Conservation Association interns for city and county-based climate change group.</t>
+  </si>
+  <si>
+    <t>To fund a CMU air pollution modeling project aimed at predicting pollution dispersion in the Mon Valley and understanding air quality under multiple meteorological conditions and emissions scenarios.</t>
+  </si>
+  <si>
+    <t>To fund Solarize Allegheny, a project promoting residential solar energy options and contacts for contractors; project managed by SmartPower, a national non-profit marketing firm for clean energy.</t>
+  </si>
+  <si>
+    <t>Support for the ACHD project incentivizing owners of indoor fireplaces to convert to natural gas instead of burning wood (vendors would receive a rebate and purchasers would get a reduced price).</t>
+  </si>
+  <si>
+    <t>To support the Southwest Pennsylvania Air Quality Partnership Lawnmower Exchange Program ($12,000 per year for two years).</t>
+  </si>
+  <si>
+    <t>To support the Carnegie Science Center Future Cities Competition ($2,000 per year for the school years 2016-2017 and 2017-2018).</t>
+  </si>
+  <si>
+    <t>To launch a new initiative ("Air-Space") to generate air quality awareness and community capacity in high priority areas throughout the County; requested by G-tech, which will partner with ACHD.</t>
+  </si>
+  <si>
+    <t>To support the Pittsburgh Regional Science &amp; Engineering Fair ($2,500 per year for 2017, 2018, and 2019).</t>
+  </si>
+  <si>
+    <t>To support placing five Student Conservation Association Sustainability Fellows in environmental organizations.</t>
+  </si>
+  <si>
+    <t>For Air Quality Program software to assist in tracking all aspects of asbestos renovation and demolition activities and stationary source enforcement; this will replace a series of spreadsheets and old software.</t>
+  </si>
+  <si>
+    <t>To fund small projects ($10k - $30k) addressing air pollution public education projects and emission reduction projects, with $150,000 going to each of the two categories.</t>
+  </si>
+  <si>
+    <t>Air Quality Program 5% operations funding allocation for the year 2017.</t>
+  </si>
+  <si>
+    <t>Construction oversight services for the potential Clack Building #1 renovation project.</t>
+  </si>
+  <si>
+    <t>Air Quality Program 5% operations funding allocation for the year 2018.</t>
+  </si>
+  <si>
+    <t>Air Quality Program 5% operations funding allocation for the year 2019.</t>
+  </si>
+  <si>
+    <t>For Air Quality Program student interns for remainder of 2018 and for 2019.</t>
+  </si>
+  <si>
+    <t>For a part-time Clean Air Fund administrator for the Air Quality Program.</t>
+  </si>
+  <si>
+    <t>For the Air Quality Program to run a half-day workshop for municipal officials on air quality topics.</t>
+  </si>
+  <si>
+    <t>To provide professional and technical support on an as-needed basis to the Air Quality Program for case analysis, data and technical support, legal support, and medical and toxicology consulting.</t>
+  </si>
+  <si>
+    <t>To fund several small projects ($10k - $30k) addressing emission reductions.</t>
+  </si>
+  <si>
+    <t>To support UPMC Children’s Hospital and Pitt GSPH developing an asthma registry for children and adolescents for surveillance and management of asthma in Allegheny County.</t>
+  </si>
+  <si>
+    <t>To fund the Allegheny County Department of Parks for the purchase of 360 landscape trees, which will be planted at designated locations in the County's Parks over a two-year period.</t>
+  </si>
+  <si>
+    <t>County Department of Public Works: for solar lighting along Corrigan Dr. in South Park.</t>
+  </si>
+  <si>
+    <t>To support the Southwest Pennsylvania Air Quality Partnership lawnmower exchange program.</t>
+  </si>
+  <si>
+    <t>To support the Carnegie Science Center Future Cities competition  ($3,000 per year for 3 years).</t>
+  </si>
+  <si>
+    <t>Carnegie Science Center Pittsburgh Regional Science and Engineering fair support ($2,500 per year for 3 years).</t>
+  </si>
+  <si>
+    <t>Air Quality Program 5% operations funding allocation for the year 2020.</t>
+  </si>
+  <si>
+    <t>For air monitoring work and equipment supporting the Air Quality Program (relocation and upgrades at the Liberty Monitor site, back-up monitoring hardware, low-cost monitors, etc.).</t>
+  </si>
+  <si>
+    <t>To update / develop software the Air Quality Program enforcement and permitting staff use.</t>
+  </si>
+  <si>
+    <t>To plant 500 trees in various locations in the Carnegie and Churchill areas.</t>
+  </si>
+  <si>
+    <t>To plant 200 street trees in various low income areas.</t>
+  </si>
+  <si>
+    <t>Air Quality Program 5% operations funding allocation for the year 2021.</t>
+  </si>
+  <si>
+    <t>To fund an RFP that will ask community-based organizations to seek small grant to conduct outreach aimed at increasing participation / sign-ups / awareness around the County's Allegheny Alerts system; titled the "Air Ambassadors  Program"; ACHD will be overseeing community partners.</t>
+  </si>
+  <si>
+    <t>To design a health impact study covering the impacts of various pollutants involving ACHD in partnership with the University of Pittsburgh, Duquesne University, and Carnegie Mellon University.</t>
+  </si>
+  <si>
+    <t>Air Quality Program 5% operations funding allocation for the year 2022.</t>
+  </si>
+  <si>
+    <t>Engage over 1000 students from 20 different schools in the Mon Valley over 2 years. Plant 1250 trees with customized tree care plan for each school. Partnership with five school districts: Bethel Park, McKeesport, Woodland Hills, West Mifflin, and South Fayette.</t>
+  </si>
+  <si>
+    <t>Annual funding for three years.</t>
+  </si>
+  <si>
+    <t>Plant and maintain 75 trees.</t>
+  </si>
+  <si>
+    <t>Professional and technical support as needed for case analysis, technical expertise, legal support, and medical and toxicological consulting.</t>
+  </si>
+  <si>
+    <t>Hire a Clean Air and Environmental Health Fund Contract grant Administrator last year to help develop new processes and outreach strategies.</t>
+  </si>
+  <si>
+    <t>Provide guidelines for individual actions to reduce exposure to pollution, provide alerts on high pollution days, and ozone and particulate forecasting for three years ($25,000 per year for 2021, 2022, and 2023).</t>
+  </si>
+  <si>
+    <t>Purchase air monitoring equipment, cover sampling analysis costs, and provide lab analysis in support of the Air Quality Program conducting a study of odor and air toxics emissions and H2S in the Mon Valley.</t>
+  </si>
+  <si>
+    <t>Online portal to be created for air quality permitting and enforcement software.</t>
+  </si>
+  <si>
+    <t>Nine organizations each work on individual projects to educate municipalities in the Mon Valley about air quality and get residents to sign up for Allegheny Alerts.</t>
+  </si>
+  <si>
+    <t>Develop an air quality forecasting program for the Mon Valley Episode Rule.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>H</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S Analysis in Allegheny County with a focus within the Mon Valley.</t>
+    </r>
+  </si>
+  <si>
+    <t>Three years of annual funding to support the Carnegie Science Center's Pittsburgh Regional Future City Competition.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replace existing 2006 diesel powered street sweeper and purchase of an equivalent electric street sweeper and installation of electric vehicle charging station. </t>
+  </si>
+  <si>
+    <t>Replace existing 2016 diesel powered garbage truck and 2014 recycling truck and purchase of an equivalent electric garbage truck and recycling truck and installation of two electric vehicle charging stations at the borough's Public Works Department.</t>
+  </si>
+  <si>
+    <t>Plant 75 caliper, balled, and burlap trees on school grounds, community parks, and right of ways within Steel Valley School District.</t>
+  </si>
+  <si>
+    <t>Plant 75 caliper, balled, and burlap trees planted on school grounds, community parks, and right of ways within the Woodland Hills School District.</t>
+  </si>
+  <si>
+    <t>Decommission and replace existing 2007 diesel-powered refuse hauler truck and replace with electric rear-load garbage packer and installation of two electric vehicle charging stations and an electrical service upgrade at the vehicle site.</t>
+  </si>
+  <si>
+    <t>Plant and maintain 50 Trees in Wilkinsburg.</t>
+  </si>
+  <si>
+    <t>Plant and maintain 45 trees in Monongahela Valley communities.</t>
+  </si>
+  <si>
+    <t>Replace eleven gas powered pieces of municipal lawn equipment with electric models.</t>
+  </si>
+  <si>
+    <t>Replace 20 gas powered pieces of municipal lawn equipment with electric models.</t>
+  </si>
+  <si>
+    <t>Replace four gas powered pieces of municipal lawn equipment with electric models for the boroughs of Braddock, East Pittsburgh, North Braddock, and Rankin.</t>
+  </si>
+  <si>
+    <t>Replace a diesel powered street sweeper with an electric model.</t>
+  </si>
+  <si>
+    <t>Support the replacement of three diesel refuse trucks with electric models and charging infrastructure.</t>
+  </si>
+  <si>
+    <t>Funding to install a 1 MWh battery storage system as part of a multi-municipality effort to install solar and battery storage systems at municipal buildings in Allegheny County.</t>
+  </si>
+  <si>
+    <t>Funding to install a solar panel and battery storage system to offset the borough building's electrical usage and to provide backup power in the event of outages.</t>
+  </si>
+  <si>
+    <t>Funding to assist the installation of solar panels, green building technologies, and tree planting at their new municipal office building.</t>
   </si>
 </sst>
 </file>
@@ -237,7 +462,7 @@
   <numFmts count="1">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -289,22 +514,23 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <vertAlign val="subscript"/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -312,11 +538,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -359,7 +594,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -378,6 +612,26 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -741,13 +995,13 @@
       <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="16" t="s">
         <v>11</v>
       </c>
       <c r="F1" s="2" t="s">
@@ -757,7 +1011,7 @@
         <v>37</v>
       </c>
       <c r="H1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -770,10 +1024,10 @@
       <c r="C2" s="10">
         <v>4000</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -783,7 +1037,7 @@
         <v>38</v>
       </c>
       <c r="H2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -796,20 +1050,20 @@
       <c r="C3" s="10">
         <v>50000</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="D3" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="18" t="s">
-        <v>56</v>
+      <c r="E3" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="17" t="s">
+        <v>55</v>
       </c>
       <c r="G3" s="15" t="s">
         <v>22</v>
       </c>
       <c r="H3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="I3" s="4"/>
     </row>
@@ -823,10 +1077,10 @@
       <c r="C4" s="10">
         <v>225000</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="E4" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F4" s="2" t="s">
@@ -836,9 +1090,9 @@
         <v>3</v>
       </c>
       <c r="H4" t="s">
-        <v>60</v>
-      </c>
-      <c r="I4" s="21"/>
+        <v>64</v>
+      </c>
+      <c r="I4" s="20"/>
     </row>
     <row r="5" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="11">
@@ -850,20 +1104,20 @@
       <c r="C5" s="10">
         <v>337600</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="D5" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G5" s="15" t="s">
         <v>23</v>
       </c>
       <c r="H5" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="I5" s="4"/>
     </row>
@@ -877,20 +1131,20 @@
       <c r="C6" s="10">
         <v>400000</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="16" t="s">
         <v>16</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G6" s="15" t="s">
         <v>39</v>
       </c>
       <c r="H6" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="I6" s="7"/>
     </row>
@@ -904,10 +1158,10 @@
       <c r="C7" s="10">
         <v>450000</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F7" s="2" t="s">
@@ -917,7 +1171,7 @@
         <v>6</v>
       </c>
       <c r="H7" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="I7" s="4"/>
     </row>
@@ -931,10 +1185,10 @@
       <c r="C8" s="10">
         <v>78000</v>
       </c>
-      <c r="D8" s="17" t="s">
+      <c r="D8" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="E8" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F8" s="2" t="s">
@@ -944,7 +1198,7 @@
         <v>9</v>
       </c>
       <c r="H8" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="I8" s="4"/>
     </row>
@@ -958,10 +1212,10 @@
       <c r="C9" s="10">
         <v>717246</v>
       </c>
-      <c r="D9" s="17" t="s">
+      <c r="D9" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="17" t="s">
+      <c r="E9" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F9" s="3" t="s">
@@ -971,7 +1225,7 @@
         <v>24</v>
       </c>
       <c r="H9" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="I9" s="4"/>
     </row>
@@ -985,10 +1239,10 @@
       <c r="C10" s="10">
         <v>180000</v>
       </c>
-      <c r="D10" s="17" t="s">
+      <c r="D10" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F10" s="2" t="s">
@@ -998,7 +1252,7 @@
         <v>25</v>
       </c>
       <c r="H10" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="I10" s="7"/>
     </row>
@@ -1009,13 +1263,13 @@
       <c r="B11" s="12">
         <v>42431</v>
       </c>
-      <c r="C11" s="19">
+      <c r="C11" s="18">
         <v>50000</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F11" s="2" t="s">
@@ -1025,7 +1279,7 @@
         <v>3</v>
       </c>
       <c r="H11" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="I11" s="7"/>
     </row>
@@ -1036,13 +1290,13 @@
       <c r="B12" s="12">
         <v>42494</v>
       </c>
-      <c r="C12" s="19">
+      <c r="C12" s="18">
         <v>24000</v>
       </c>
-      <c r="D12" s="17" t="s">
+      <c r="D12" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E12" s="17" t="s">
+      <c r="E12" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F12" s="2" t="s">
@@ -1052,7 +1306,7 @@
         <v>4</v>
       </c>
       <c r="H12" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="I12" s="7"/>
     </row>
@@ -1063,13 +1317,13 @@
       <c r="B13" s="12">
         <v>42564</v>
       </c>
-      <c r="C13" s="19">
+      <c r="C13" s="18">
         <v>4000</v>
       </c>
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="E13" s="17" t="s">
+      <c r="E13" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F13" s="2" t="s">
@@ -1079,7 +1333,7 @@
         <v>38</v>
       </c>
       <c r="H13" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1089,23 +1343,23 @@
       <c r="B14" s="12">
         <v>43041</v>
       </c>
-      <c r="C14" s="19">
+      <c r="C14" s="18">
         <v>75900</v>
       </c>
-      <c r="D14" s="17" t="s">
+      <c r="D14" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="15" t="s">
+      <c r="G14" s="27" t="s">
         <v>3</v>
       </c>
       <c r="H14" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="I14" s="4"/>
     </row>
@@ -1119,20 +1373,20 @@
       <c r="C15" s="10">
         <v>7500</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="D15" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="E15" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G15" s="15" t="s">
+      <c r="G15" s="27" t="s">
         <v>7</v>
       </c>
       <c r="H15" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="I15" s="4"/>
     </row>
@@ -1146,20 +1400,20 @@
       <c r="C16" s="10">
         <v>65000</v>
       </c>
-      <c r="D16" s="17" t="s">
+      <c r="D16" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="E16" s="17" t="s">
+      <c r="E16" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G16" s="15" t="s">
+      <c r="G16" s="27" t="s">
         <v>9</v>
       </c>
       <c r="H16" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1172,20 +1426,20 @@
       <c r="C17" s="10">
         <v>45000</v>
       </c>
-      <c r="D17" s="17" t="s">
+      <c r="D17" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E17" s="17" t="s">
+      <c r="E17" s="16" t="s">
         <v>19</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G17" s="15" t="s">
+      <c r="G17" s="27" t="s">
         <v>6</v>
       </c>
       <c r="H17" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="I17" s="7"/>
     </row>
@@ -1199,20 +1453,20 @@
       <c r="C18" s="10">
         <v>300000</v>
       </c>
-      <c r="D18" s="17" t="s">
+      <c r="D18" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="E18" s="17" t="s">
+      <c r="E18" s="16" t="s">
         <v>15</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G18" s="16" t="s">
-        <v>63</v>
+      <c r="G18" s="27" t="s">
+        <v>61</v>
       </c>
       <c r="H18" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="I18" s="7"/>
     </row>
@@ -1226,22 +1480,22 @@
       <c r="C19" s="10">
         <v>558242</v>
       </c>
-      <c r="D19" s="17" t="s">
+      <c r="D19" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E19" s="17" t="s">
+      <c r="E19" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="15" t="s">
+      <c r="G19" s="27" t="s">
         <v>6</v>
       </c>
       <c r="H19" t="s">
-        <v>60</v>
-      </c>
-      <c r="I19" s="22"/>
+        <v>79</v>
+      </c>
+      <c r="I19" s="21"/>
     </row>
     <row r="20" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="11">
@@ -1253,20 +1507,20 @@
       <c r="C20" s="10">
         <v>66000</v>
       </c>
-      <c r="D20" s="17" t="s">
+      <c r="D20" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E20" s="17" t="s">
+      <c r="E20" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="15" t="s">
+      <c r="G20" s="27" t="s">
         <v>6</v>
       </c>
       <c r="H20" t="s">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="I20" s="4"/>
     </row>
@@ -1280,20 +1534,20 @@
       <c r="C21" s="10">
         <v>579703</v>
       </c>
-      <c r="D21" s="17" t="s">
+      <c r="D21" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E21" s="17" t="s">
+      <c r="E21" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G21" s="15" t="s">
+      <c r="G21" s="27" t="s">
         <v>6</v>
       </c>
       <c r="H21" t="s">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="I21" s="4"/>
     </row>
@@ -1307,20 +1561,20 @@
       <c r="C22" s="10">
         <v>546017</v>
       </c>
-      <c r="D22" s="17" t="s">
+      <c r="D22" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E22" s="17" t="s">
+      <c r="E22" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G22" s="15" t="s">
+      <c r="G22" s="27" t="s">
         <v>6</v>
       </c>
       <c r="H22" t="s">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="I22" s="4"/>
     </row>
@@ -1334,20 +1588,20 @@
       <c r="C23" s="10">
         <v>60000</v>
       </c>
-      <c r="D23" s="17" t="s">
+      <c r="D23" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E23" s="17" t="s">
+      <c r="E23" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G23" s="15" t="s">
+      <c r="G23" s="27" t="s">
         <v>6</v>
       </c>
       <c r="H23" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="I23" s="4"/>
     </row>
@@ -1361,20 +1615,20 @@
       <c r="C24" s="10">
         <v>24765</v>
       </c>
-      <c r="D24" s="17" t="s">
+      <c r="D24" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E24" s="17" t="s">
+      <c r="E24" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G24" s="15" t="s">
+      <c r="G24" s="27" t="s">
         <v>6</v>
       </c>
       <c r="H24" t="s">
-        <v>60</v>
+        <v>84</v>
       </c>
       <c r="I24" s="4"/>
     </row>
@@ -1388,20 +1642,20 @@
       <c r="C25" s="10">
         <v>15000</v>
       </c>
-      <c r="D25" s="17" t="s">
+      <c r="D25" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E25" s="17" t="s">
+      <c r="E25" s="16" t="s">
         <v>20</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G25" s="15" t="s">
+      <c r="G25" s="27" t="s">
         <v>6</v>
       </c>
       <c r="H25" t="s">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="I25" s="4"/>
     </row>
@@ -1415,20 +1669,20 @@
       <c r="C26" s="10">
         <v>120000</v>
       </c>
-      <c r="D26" s="17" t="s">
+      <c r="D26" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E26" s="17" t="s">
+      <c r="E26" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G26" s="15" t="s">
+      <c r="G26" s="27" t="s">
         <v>6</v>
       </c>
       <c r="H26" t="s">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="I26" s="5"/>
     </row>
@@ -1442,20 +1696,20 @@
       <c r="C27" s="10">
         <v>150000</v>
       </c>
-      <c r="D27" s="17" t="s">
+      <c r="D27" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="E27" s="17" t="s">
+      <c r="E27" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G27" s="16" t="s">
-        <v>63</v>
+      <c r="G27" s="27" t="s">
+        <v>61</v>
       </c>
       <c r="H27" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="I27" s="8"/>
     </row>
@@ -1469,20 +1723,20 @@
       <c r="C28" s="10">
         <v>300000</v>
       </c>
-      <c r="D28" s="17" t="s">
+      <c r="D28" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="E28" s="17" t="s">
+      <c r="E28" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G28" s="6" t="s">
+      <c r="G28" s="28" t="s">
         <v>40</v>
       </c>
       <c r="H28" t="s">
-        <v>60</v>
+        <v>88</v>
       </c>
       <c r="I28" s="5"/>
     </row>
@@ -1499,17 +1753,17 @@
       <c r="D29" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="E29" s="17" t="s">
+      <c r="E29" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F29" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="G29" s="15" t="s">
+      <c r="G29" s="27" t="s">
         <v>27</v>
       </c>
       <c r="H29" t="s">
-        <v>60</v>
+        <v>89</v>
       </c>
       <c r="I29" s="5"/>
     </row>
@@ -1523,20 +1777,20 @@
       <c r="C30" s="10">
         <v>627100</v>
       </c>
-      <c r="D30" s="17" t="s">
+      <c r="D30" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="E30" s="17" t="s">
+      <c r="E30" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="G30" s="15" t="s">
+      <c r="G30" s="27" t="s">
         <v>3</v>
       </c>
       <c r="H30" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="I30" s="8"/>
     </row>
@@ -1550,20 +1804,20 @@
       <c r="C31" s="10">
         <v>25000</v>
       </c>
-      <c r="D31" s="17" t="s">
+      <c r="D31" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E31" s="17" t="s">
+      <c r="E31" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="14" t="s">
+      <c r="G31" s="29" t="s">
         <v>4</v>
       </c>
       <c r="H31" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="I31" s="4"/>
     </row>
@@ -1577,20 +1831,20 @@
       <c r="C32" s="10">
         <v>9000</v>
       </c>
-      <c r="D32" s="17" t="s">
+      <c r="D32" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="E32" s="17" t="s">
+      <c r="E32" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G32" s="2" t="s">
+      <c r="G32" s="30" t="s">
         <v>38</v>
       </c>
       <c r="H32" t="s">
-        <v>60</v>
+        <v>92</v>
       </c>
       <c r="I32" s="5"/>
     </row>
@@ -1604,20 +1858,20 @@
       <c r="C33" s="10">
         <v>7500</v>
       </c>
-      <c r="D33" s="17" t="s">
+      <c r="D33" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="E33" s="17" t="s">
+      <c r="E33" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F33" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G33" s="2" t="s">
+      <c r="G33" s="30" t="s">
         <v>38</v>
       </c>
       <c r="H33" t="s">
-        <v>60</v>
+        <v>93</v>
       </c>
       <c r="I33" s="5"/>
     </row>
@@ -1631,20 +1885,20 @@
       <c r="C34" s="10">
         <v>592822</v>
       </c>
-      <c r="D34" s="17" t="s">
+      <c r="D34" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E34" s="17" t="s">
+      <c r="E34" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G34" s="15" t="s">
+      <c r="G34" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="H34" t="s">
-        <v>60</v>
+      <c r="H34" s="23" t="s">
+        <v>94</v>
       </c>
       <c r="I34" s="5"/>
     </row>
@@ -1658,20 +1912,20 @@
       <c r="C35" s="10">
         <v>384000</v>
       </c>
-      <c r="D35" s="17" t="s">
+      <c r="D35" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E35" s="17" t="s">
+      <c r="E35" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G35" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="H35" t="s">
+      <c r="G35" s="27" t="s">
         <v>60</v>
+      </c>
+      <c r="H35" s="23" t="s">
+        <v>95</v>
       </c>
       <c r="I35" s="5"/>
     </row>
@@ -1685,10 +1939,10 @@
       <c r="C36" s="10">
         <v>500000</v>
       </c>
-      <c r="D36" s="17" t="s">
+      <c r="D36" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E36" s="17" t="s">
+      <c r="E36" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F36" s="2" t="s">
@@ -1697,8 +1951,8 @@
       <c r="G36" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="H36" t="s">
-        <v>60</v>
+      <c r="H36" s="24" t="s">
+        <v>86</v>
       </c>
       <c r="I36" s="5"/>
     </row>
@@ -1712,10 +1966,10 @@
       <c r="C37" s="10">
         <v>210000</v>
       </c>
-      <c r="D37" s="17" t="s">
+      <c r="D37" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E37" s="17" t="s">
+      <c r="E37" s="16" t="s">
         <v>19</v>
       </c>
       <c r="F37" s="2" t="s">
@@ -1724,8 +1978,8 @@
       <c r="G37" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="H37" t="s">
-        <v>60</v>
+      <c r="H37" s="23" t="s">
+        <v>96</v>
       </c>
       <c r="I37" s="8"/>
     </row>
@@ -1739,10 +1993,10 @@
       <c r="C38" s="10">
         <v>59560</v>
       </c>
-      <c r="D38" s="17" t="s">
+      <c r="D38" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="E38" s="17" t="s">
+      <c r="E38" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F38" s="6" t="s">
@@ -1751,8 +2005,8 @@
       <c r="G38" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="H38" t="s">
-        <v>60</v>
+      <c r="H38" s="23" t="s">
+        <v>97</v>
       </c>
       <c r="I38" s="5"/>
     </row>
@@ -1766,20 +2020,20 @@
       <c r="C39" s="10">
         <v>98000</v>
       </c>
-      <c r="D39" s="17" t="s">
+      <c r="D39" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="E39" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="F39" s="23" t="s">
+      <c r="E39" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="F39" s="22" t="s">
         <v>26</v>
       </c>
       <c r="G39" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="H39" t="s">
-        <v>60</v>
+      <c r="H39" s="23" t="s">
+        <v>98</v>
       </c>
       <c r="I39" s="5"/>
     </row>
@@ -1796,7 +2050,7 @@
       <c r="D40" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="E40" s="17" t="s">
+      <c r="E40" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F40" s="2" t="s">
@@ -1805,8 +2059,8 @@
       <c r="G40" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="H40" t="s">
-        <v>60</v>
+      <c r="H40" s="23" t="s">
+        <v>99</v>
       </c>
       <c r="I40" s="5"/>
     </row>
@@ -1820,10 +2074,10 @@
       <c r="C41" s="10">
         <v>200000</v>
       </c>
-      <c r="D41" s="17" t="s">
+      <c r="D41" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="E41" s="17" t="s">
+      <c r="E41" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F41" s="2" t="s">
@@ -1832,8 +2086,8 @@
       <c r="G41" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="H41" t="s">
-        <v>60</v>
+      <c r="H41" s="23" t="s">
+        <v>100</v>
       </c>
       <c r="I41" s="5"/>
     </row>
@@ -1847,10 +2101,10 @@
       <c r="C42" s="10">
         <v>30000</v>
       </c>
-      <c r="D42" s="17" t="s">
+      <c r="D42" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="E42" s="17" t="s">
+      <c r="E42" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F42" s="2" t="s">
@@ -1859,8 +2113,8 @@
       <c r="G42" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="H42" t="s">
-        <v>60</v>
+      <c r="H42" s="23" t="s">
+        <v>101</v>
       </c>
       <c r="I42" s="5"/>
     </row>
@@ -1874,10 +2128,10 @@
       <c r="C43" s="10">
         <v>539125</v>
       </c>
-      <c r="D43" s="17" t="s">
+      <c r="D43" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E43" s="17" t="s">
+      <c r="E43" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F43" s="2" t="s">
@@ -1886,8 +2140,8 @@
       <c r="G43" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="H43" t="s">
-        <v>60</v>
+      <c r="H43" s="23" t="s">
+        <v>102</v>
       </c>
       <c r="I43" s="5"/>
     </row>
@@ -1901,7 +2155,7 @@
       <c r="C44" s="10">
         <v>99995</v>
       </c>
-      <c r="D44" s="17" t="s">
+      <c r="D44" s="16" t="s">
         <v>13</v>
       </c>
       <c r="E44" s="11" t="s">
@@ -1913,8 +2167,8 @@
       <c r="G44" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="H44" t="s">
-        <v>60</v>
+      <c r="H44" s="24" t="s">
+        <v>103</v>
       </c>
       <c r="I44" s="5"/>
     </row>
@@ -1928,10 +2182,10 @@
       <c r="C45" s="10">
         <v>15000</v>
       </c>
-      <c r="D45" s="17" t="s">
+      <c r="D45" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="E45" s="17" t="s">
+      <c r="E45" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F45" s="2" t="s">
@@ -1940,8 +2194,8 @@
       <c r="G45" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="H45" t="s">
-        <v>60</v>
+      <c r="H45" s="24" t="s">
+        <v>104</v>
       </c>
       <c r="I45" s="5"/>
     </row>
@@ -1955,10 +2209,10 @@
       <c r="C46" s="10">
         <v>98000</v>
       </c>
-      <c r="D46" s="17" t="s">
+      <c r="D46" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="E46" s="17" t="s">
+      <c r="E46" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F46" s="6" t="s">
@@ -1967,8 +2221,8 @@
       <c r="G46" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="H46" t="s">
-        <v>60</v>
+      <c r="H46" s="24" t="s">
+        <v>105</v>
       </c>
       <c r="I46" s="5"/>
     </row>
@@ -1982,10 +2236,10 @@
       <c r="C47" s="10">
         <v>500000</v>
       </c>
-      <c r="D47" s="17" t="s">
+      <c r="D47" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E47" s="17" t="s">
+      <c r="E47" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F47" s="2" t="s">
@@ -1994,8 +2248,8 @@
       <c r="G47" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="H47" t="s">
-        <v>60</v>
+      <c r="H47" s="24" t="s">
+        <v>106</v>
       </c>
       <c r="I47" s="5"/>
     </row>
@@ -2009,10 +2263,10 @@
       <c r="C48" s="10">
         <v>55000</v>
       </c>
-      <c r="D48" s="17" t="s">
+      <c r="D48" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E48" s="17" t="s">
+      <c r="E48" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F48" s="2" t="s">
@@ -2021,8 +2275,8 @@
       <c r="G48" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="H48" t="s">
-        <v>60</v>
+      <c r="H48" s="24" t="s">
+        <v>107</v>
       </c>
       <c r="I48" s="5"/>
     </row>
@@ -2036,10 +2290,10 @@
       <c r="C49" s="10">
         <v>75000</v>
       </c>
-      <c r="D49" s="17" t="s">
+      <c r="D49" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E49" s="17" t="s">
+      <c r="E49" s="16" t="s">
         <v>20</v>
       </c>
       <c r="F49" s="2" t="s">
@@ -2048,8 +2302,8 @@
       <c r="G49" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="H49" t="s">
-        <v>60</v>
+      <c r="H49" s="24" t="s">
+        <v>108</v>
       </c>
       <c r="I49" s="5"/>
     </row>
@@ -2063,10 +2317,10 @@
       <c r="C50" s="10">
         <v>340554</v>
       </c>
-      <c r="D50" s="17" t="s">
+      <c r="D50" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E50" s="17" t="s">
+      <c r="E50" s="16" t="s">
         <v>18</v>
       </c>
       <c r="F50" s="2" t="s">
@@ -2075,8 +2329,8 @@
       <c r="G50" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="H50" t="s">
-        <v>60</v>
+      <c r="H50" s="24" t="s">
+        <v>109</v>
       </c>
       <c r="I50" s="5"/>
     </row>
@@ -2090,10 +2344,10 @@
       <c r="C51" s="10">
         <v>548725</v>
       </c>
-      <c r="D51" s="17" t="s">
+      <c r="D51" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E51" s="17" t="s">
+      <c r="E51" s="16" t="s">
         <v>19</v>
       </c>
       <c r="F51" s="2" t="s">
@@ -2102,10 +2356,10 @@
       <c r="G51" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="H51" t="s">
-        <v>60</v>
-      </c>
-      <c r="I51" s="23"/>
+      <c r="H51" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="I51" s="22"/>
     </row>
     <row r="52" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" s="11">
@@ -2117,22 +2371,22 @@
       <c r="C52" s="10">
         <v>200000</v>
       </c>
-      <c r="D52" s="17" t="s">
+      <c r="D52" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="E52" s="17" t="s">
+      <c r="E52" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F52" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="G52" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="H52" t="s">
-        <v>60</v>
-      </c>
-      <c r="I52" s="23"/>
+      <c r="G52" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="H52" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="I52" s="22"/>
     </row>
     <row r="53" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A53" s="11">
@@ -2144,10 +2398,10 @@
       <c r="C53" s="13">
         <v>9941</v>
       </c>
-      <c r="D53" s="17" t="s">
+      <c r="D53" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="E53" s="17" t="s">
+      <c r="E53" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F53" s="3" t="s">
@@ -2156,12 +2410,12 @@
       <c r="G53" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="H53" t="s">
-        <v>60</v>
-      </c>
-      <c r="I53" s="23"/>
-    </row>
-    <row r="54" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="H53" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="I53" s="22"/>
+    </row>
+    <row r="54" spans="1:9" ht="18" x14ac:dyDescent="0.2">
       <c r="A54" s="11">
         <v>2021</v>
       </c>
@@ -2171,10 +2425,10 @@
       <c r="C54" s="13">
         <v>69956</v>
       </c>
-      <c r="D54" s="17" t="s">
+      <c r="D54" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="E54" s="17" t="s">
+      <c r="E54" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F54" s="3" t="s">
@@ -2183,10 +2437,10 @@
       <c r="G54" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="H54" t="s">
-        <v>60</v>
-      </c>
-      <c r="I54" s="23"/>
+      <c r="H54" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="I54" s="22"/>
     </row>
     <row r="55" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A55" s="11">
@@ -2198,10 +2452,10 @@
       <c r="C55" s="10">
         <v>9000</v>
       </c>
-      <c r="D55" s="17" t="s">
+      <c r="D55" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="E55" s="17" t="s">
+      <c r="E55" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F55" s="2" t="s">
@@ -2210,8 +2464,8 @@
       <c r="G55" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="H55" t="s">
-        <v>60</v>
+      <c r="H55" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="I55" s="5"/>
     </row>
@@ -2225,20 +2479,20 @@
       <c r="C56" s="10">
         <v>750000</v>
       </c>
-      <c r="D56" s="17" t="s">
+      <c r="D56" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E56" s="17" t="s">
+      <c r="E56" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F56" s="3" t="s">
         <v>44</v>
       </c>
       <c r="G56" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="H56" t="s">
-        <v>60</v>
+        <v>59</v>
+      </c>
+      <c r="H56" s="24" t="s">
+        <v>115</v>
       </c>
       <c r="I56" s="8"/>
     </row>
@@ -2255,7 +2509,7 @@
       <c r="D57" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="E57" s="17" t="s">
+      <c r="E57" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F57" s="3" t="s">
@@ -2264,10 +2518,10 @@
       <c r="G57" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="H57" t="s">
-        <v>60</v>
-      </c>
-      <c r="I57" s="20"/>
+      <c r="H57" s="24" t="s">
+        <v>116</v>
+      </c>
+      <c r="I57" s="19"/>
     </row>
     <row r="58" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A58" s="11">
@@ -2279,10 +2533,10 @@
       <c r="C58" s="10">
         <v>46000</v>
       </c>
-      <c r="D58" s="17" t="s">
+      <c r="D58" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="E58" s="17" t="s">
+      <c r="E58" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F58" s="6" t="s">
@@ -2291,8 +2545,8 @@
       <c r="G58" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="H58" t="s">
-        <v>60</v>
+      <c r="H58" s="24" t="s">
+        <v>117</v>
       </c>
       <c r="I58" s="5"/>
     </row>
@@ -2306,10 +2560,10 @@
       <c r="C59" s="10">
         <v>46000</v>
       </c>
-      <c r="D59" s="17" t="s">
+      <c r="D59" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="E59" s="17" t="s">
+      <c r="E59" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F59" s="6" t="s">
@@ -2318,8 +2572,8 @@
       <c r="G59" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="H59" t="s">
-        <v>60</v>
+      <c r="H59" s="24" t="s">
+        <v>118</v>
       </c>
       <c r="I59" s="5"/>
     </row>
@@ -2333,10 +2587,10 @@
       <c r="C60" s="10">
         <v>748339</v>
       </c>
-      <c r="D60" s="17" t="s">
+      <c r="D60" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E60" s="17" t="s">
+      <c r="E60" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F60" s="6" t="s">
@@ -2345,8 +2599,8 @@
       <c r="G60" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="H60" t="s">
-        <v>60</v>
+      <c r="H60" s="24" t="s">
+        <v>119</v>
       </c>
       <c r="I60" s="8"/>
     </row>
@@ -2360,10 +2614,10 @@
       <c r="C61" s="10">
         <v>46000</v>
       </c>
-      <c r="D61" s="17" t="s">
+      <c r="D61" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="E61" s="17" t="s">
+      <c r="E61" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F61" s="3" t="s">
@@ -2372,8 +2626,8 @@
       <c r="G61" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="H61" t="s">
-        <v>60</v>
+      <c r="H61" s="24" t="s">
+        <v>120</v>
       </c>
       <c r="I61" s="5"/>
     </row>
@@ -2387,10 +2641,10 @@
       <c r="C62" s="10">
         <v>46000</v>
       </c>
-      <c r="D62" s="17" t="s">
+      <c r="D62" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="E62" s="17" t="s">
+      <c r="E62" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F62" s="3" t="s">
@@ -2399,8 +2653,8 @@
       <c r="G62" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="H62" t="s">
-        <v>60</v>
+      <c r="H62" s="24" t="s">
+        <v>121</v>
       </c>
       <c r="I62" s="5"/>
     </row>
@@ -2414,10 +2668,10 @@
       <c r="C63" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D63" s="17" t="s">
+      <c r="D63" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E63" s="17" t="s">
+      <c r="E63" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F63" s="6" t="s">
@@ -2426,8 +2680,8 @@
       <c r="G63" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="H63" t="s">
-        <v>60</v>
+      <c r="H63" s="24" t="s">
+        <v>122</v>
       </c>
       <c r="I63" s="8"/>
     </row>
@@ -2441,10 +2695,10 @@
       <c r="C64" s="10">
         <v>43272</v>
       </c>
-      <c r="D64" s="17" t="s">
+      <c r="D64" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E64" s="17" t="s">
+      <c r="E64" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F64" s="3" t="s">
@@ -2453,8 +2707,8 @@
       <c r="G64" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="H64" t="s">
-        <v>60</v>
+      <c r="H64" s="24" t="s">
+        <v>123</v>
       </c>
       <c r="I64" s="8"/>
     </row>
@@ -2468,22 +2722,22 @@
       <c r="C65" s="10">
         <v>75000</v>
       </c>
-      <c r="D65" s="17" t="s">
+      <c r="D65" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E65" s="17" t="s">
+      <c r="E65" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F65" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G65" s="20" t="s">
+      <c r="G65" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="H65" t="s">
-        <v>60</v>
-      </c>
-      <c r="I65" s="20"/>
+      <c r="H65" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="I65" s="19"/>
     </row>
     <row r="66" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A66" s="11">
@@ -2495,10 +2749,10 @@
       <c r="C66" s="10">
         <v>800000</v>
       </c>
-      <c r="D66" s="17" t="s">
+      <c r="D66" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E66" s="17" t="s">
+      <c r="E66" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F66" s="3" t="s">
@@ -2507,8 +2761,8 @@
       <c r="G66" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="H66" t="s">
-        <v>60</v>
+      <c r="H66" s="24" t="s">
+        <v>125</v>
       </c>
       <c r="I66" s="8"/>
     </row>
@@ -2522,10 +2776,10 @@
       <c r="C67" s="10">
         <v>186789</v>
       </c>
-      <c r="D67" s="17" t="s">
+      <c r="D67" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E67" s="17" t="s">
+      <c r="E67" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F67" s="3" t="s">
@@ -2534,8 +2788,8 @@
       <c r="G67" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="H67" t="s">
-        <v>60</v>
+      <c r="H67" s="24" t="s">
+        <v>126</v>
       </c>
       <c r="I67" s="8"/>
     </row>
@@ -2549,10 +2803,10 @@
       <c r="C68" s="10">
         <v>997450</v>
       </c>
-      <c r="D68" s="17" t="s">
+      <c r="D68" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="E68" s="17" t="s">
+      <c r="E68" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F68" s="3" t="s">
@@ -2561,8 +2815,8 @@
       <c r="G68" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="H68" t="s">
-        <v>60</v>
+      <c r="H68" s="24" t="s">
+        <v>127</v>
       </c>
       <c r="I68" s="8"/>
     </row>
@@ -2576,10 +2830,10 @@
       <c r="C69" s="10">
         <v>1000000</v>
       </c>
-      <c r="D69" s="17" t="s">
+      <c r="D69" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="E69" s="17" t="s">
+      <c r="E69" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F69" s="3" t="s">
@@ -2588,8 +2842,8 @@
       <c r="G69" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="H69" t="s">
-        <v>60</v>
+      <c r="H69" s="24" t="s">
+        <v>128</v>
       </c>
       <c r="I69" s="8"/>
     </row>
@@ -2603,10 +2857,10 @@
       <c r="C70" s="10">
         <v>500000</v>
       </c>
-      <c r="D70" s="17" t="s">
+      <c r="D70" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="E70" s="17" t="s">
+      <c r="E70" s="16" t="s">
         <v>15</v>
       </c>
       <c r="F70" s="3" t="s">
@@ -2615,8 +2869,8 @@
       <c r="G70" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="H70" t="s">
-        <v>60</v>
+      <c r="H70" s="26" t="s">
+        <v>129</v>
       </c>
       <c r="I70" s="5"/>
     </row>

</xml_diff>